<commit_message>
finised the test for investment account
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_investment_account.xlsx
+++ b/tests/A02_pixell_test_plan_investment_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Updated Assignments ISD\assignment_02\given_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\OneDrive\Desktop\Documents\rrc-ploytech\semi-2\ISD 2327 assignments\Assignment_1_harshdeep_bhinder\isd_project_harshdeep\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6AEFC8-F3D7-467B-9A12-00596A3BA98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4037F805-2CF1-434D-93CA-A55A0154B78B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="25185" windowHeight="13845" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -246,6 +246,12 @@
   </si>
   <si>
     <t>date created exactly 10 years ago.</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>Column1</t>
   </si>
 </sst>
 </file>
@@ -332,7 +338,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -548,11 +554,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -608,11 +640,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -820,14 +876,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B0B8C9F-A34D-46F3-9066-19FDAF76B033}" name="Table1" displayName="Table1" ref="B6:G32" totalsRowShown="0" headerRowDxfId="6">
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B4BB882C-2019-4F87-8900-426FA9A11FFB}" name="Test Case ID" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{1904C92F-9639-4229-AA4E-4C4DEAF21EEE}" name="Method being Tested" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{4E480EB6-99FB-4F51-98B5-D5BE13327E8C}" name="Condition being Tested" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{5381561B-09C5-439D-999E-CD8E013F9561}" name="Preconditions" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{645704DE-22F5-4239-BEB6-F4252A1F2823}" name="Method Inputs" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{101F480E-86C3-4E60-AA1E-2FCAD389E35F}" name="Expected Result" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B0B8C9F-A34D-46F3-9066-19FDAF76B033}" name="Table1" displayName="Table1" ref="B6:H32" totalsRowShown="0" headerRowDxfId="7">
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B4BB882C-2019-4F87-8900-426FA9A11FFB}" name="Test Case ID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{1904C92F-9639-4229-AA4E-4C4DEAF21EEE}" name="Method being Tested" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{4E480EB6-99FB-4F51-98B5-D5BE13327E8C}" name="Condition being Tested" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{5381561B-09C5-439D-999E-CD8E013F9561}" name="Preconditions" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{645704DE-22F5-4239-BEB6-F4252A1F2823}" name="Method Inputs" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{101F480E-86C3-4E60-AA1E-2FCAD389E35F}" name="Expected Result" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{88C6697F-A3F5-4D52-9130-6C1E4BFCC9A8}" name="Column1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1150,19 +1207,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DADEBCC4-BB44-48CD-B9AB-1E2FD3EE0EEB}">
-  <dimension ref="B1:G34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:H34"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" customWidth="1"/>
-    <col min="6" max="6" width="28.28515625" customWidth="1"/>
-    <col min="7" max="7" width="49.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" customWidth="1"/>
+    <col min="5" max="5" width="27.109375" customWidth="1"/>
+    <col min="6" max="6" width="28.33203125" customWidth="1"/>
+    <col min="7" max="7" width="49.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:7" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="1.45">
+    <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:8" ht="73.2" customHeight="1" thickBot="1" x14ac:dyDescent="1.8">
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -1174,14 +1231,14 @@
       <c r="F2" s="16"/>
       <c r="G2" s="16"/>
     </row>
-    <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="18"/>
     </row>
-    <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
@@ -1190,10 +1247,10 @@
       </c>
       <c r="D4" s="20"/>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="s">
         <v>0</v>
       </c>
@@ -1212,8 +1269,11 @@
       <c r="G6" s="9" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H6" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="11">
         <v>1</v>
       </c>
@@ -1226,8 +1286,11 @@
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
-    </row>
-    <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H7" s="23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="3">
         <v>2</v>
       </c>
@@ -1240,8 +1303,9 @@
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="13"/>
-    </row>
-    <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="11">
         <v>3</v>
       </c>
@@ -1254,8 +1318,9 @@
       <c r="E9" s="12"/>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
-    </row>
-    <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="11">
         <v>4</v>
       </c>
@@ -1268,8 +1333,9 @@
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
-    </row>
-    <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="11">
         <v>5</v>
       </c>
@@ -1282,8 +1348,9 @@
       <c r="E11" s="12"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
-    </row>
-    <row r="12" spans="2:7" ht="74.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="2:8" ht="74.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="3">
         <v>6</v>
       </c>
@@ -1296,8 +1363,9 @@
       <c r="E12" s="12"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
-    </row>
-    <row r="13" spans="2:7" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="2:8" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="11">
         <v>7</v>
       </c>
@@ -1310,8 +1378,9 @@
       <c r="E13" s="12"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H13" s="14"/>
+    </row>
+    <row r="14" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="11">
         <v>8</v>
       </c>
@@ -1320,8 +1389,9 @@
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H14" s="14"/>
+    </row>
+    <row r="15" spans="2:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="11">
         <v>9</v>
       </c>
@@ -1330,8 +1400,9 @@
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H15" s="14"/>
+    </row>
+    <row r="16" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="3">
         <v>10</v>
       </c>
@@ -1340,8 +1411,9 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H16" s="14"/>
+    </row>
+    <row r="17" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="11">
         <v>11</v>
       </c>
@@ -1350,8 +1422,9 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H17" s="14"/>
+    </row>
+    <row r="18" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="11">
         <v>12</v>
       </c>
@@ -1360,8 +1433,9 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H18" s="14"/>
+    </row>
+    <row r="19" spans="2:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11">
         <v>13</v>
       </c>
@@ -1370,8 +1444,9 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H19" s="14"/>
+    </row>
+    <row r="20" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="3">
         <v>14</v>
       </c>
@@ -1380,8 +1455,9 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H20" s="14"/>
+    </row>
+    <row r="21" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="11">
         <v>15</v>
       </c>
@@ -1390,8 +1466,9 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H21" s="14"/>
+    </row>
+    <row r="22" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="11">
         <v>16</v>
       </c>
@@ -1400,8 +1477,9 @@
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
-    </row>
-    <row r="23" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H22" s="14"/>
+    </row>
+    <row r="23" spans="2:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="11">
         <v>17</v>
       </c>
@@ -1410,8 +1488,9 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H23" s="14"/>
+    </row>
+    <row r="24" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="3">
         <v>18</v>
       </c>
@@ -1420,8 +1499,9 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-    </row>
-    <row r="25" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H24" s="14"/>
+    </row>
+    <row r="25" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="11">
         <v>19</v>
       </c>
@@ -1430,8 +1510,9 @@
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
-    </row>
-    <row r="26" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H25" s="14"/>
+    </row>
+    <row r="26" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="11">
         <v>20</v>
       </c>
@@ -1440,8 +1521,9 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
-    </row>
-    <row r="27" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H26" s="14"/>
+    </row>
+    <row r="27" spans="2:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="11">
         <v>21</v>
       </c>
@@ -1450,8 +1532,9 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
-    </row>
-    <row r="28" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H27" s="14"/>
+    </row>
+    <row r="28" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="3">
         <v>22</v>
       </c>
@@ -1460,8 +1543,9 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
-    </row>
-    <row r="29" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H28" s="14"/>
+    </row>
+    <row r="29" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11">
         <v>23</v>
       </c>
@@ -1470,8 +1554,9 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
-    </row>
-    <row r="30" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H29" s="14"/>
+    </row>
+    <row r="30" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="11">
         <v>24</v>
       </c>
@@ -1480,8 +1565,9 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
-    </row>
-    <row r="31" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H30" s="14"/>
+    </row>
+    <row r="31" spans="2:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="11">
         <v>25</v>
       </c>
@@ -1490,8 +1576,9 @@
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
-    </row>
-    <row r="32" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H31" s="14"/>
+    </row>
+    <row r="32" spans="2:8" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="3">
         <v>26</v>
       </c>
@@ -1500,8 +1587,9 @@
       <c r="E32" s="5"/>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H32" s="24"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B34" s="21" t="s">
         <v>6</v>
       </c>

</xml_diff>